<commit_message>
Update PINKI BHOI (S.No.478): Hall Ticket 147203098->2608LPT031, Mobile 9765213553
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -28451,7 +28451,7 @@
       </c>
       <c r="C438" t="inlineStr">
         <is>
-          <t>147203098</t>
+          <t>2608LPT031</t>
         </is>
       </c>
       <c r="D438" t="inlineStr">
@@ -28464,7 +28464,6 @@
           <t>202752073337</t>
         </is>
       </c>
-      <c r="F438" t="inlineStr"/>
       <c r="G438" t="inlineStr">
         <is>
           <t>FEMALE</t>
@@ -28475,7 +28474,11 @@
           <t>PGT ENGLISH</t>
         </is>
       </c>
-      <c r="I438" t="inlineStr"/>
+      <c r="I438" t="inlineStr">
+        <is>
+          <t>9765213553</t>
+        </is>
+      </c>
       <c r="J438" t="inlineStr">
         <is>
           <t>EMRS MELIAPUTTI, VILL-MELIAPUTTI, DIST.- SRIKAKULAM, 532215 AP</t>

</xml_diff>